<commit_message>
docs: apply standardized excel formatting from MP-01 to MP-02 through MP-06 content cells
</commit_message>
<xml_diff>
--- a/report/mearsuring-profile/MP-02_Drive_Fast_Travel_Steer.xlsx
+++ b/report/mearsuring-profile/MP-02_Drive_Fast_Travel_Steer.xlsx
@@ -590,8 +590,15 @@
   </sheetPr>
   <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18.28515625" customWidth="1" min="1" max="1"/>
+    <col width="42.7109375" customWidth="1" min="2" max="2"/>
+    <col width="29.28515625" customWidth="1" min="4" max="4"/>
+    <col width="13.42578125" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>▶  MP-02 Drive Fast - Travel &amp; Steer Performance  |  Tests: LOAD-004, LOAD-005, LOAD-013, PERF-003, PERF-005, PERF-006, PERF-007
@@ -651,7 +658,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>current_travelA</t>
@@ -695,7 +702,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
+    <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>current_travelB</t>
@@ -739,7 +746,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1">
+    <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>current_travelC</t>
@@ -783,7 +790,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>current_travelD</t>
@@ -827,7 +834,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>batt_voltage_travelA</t>
@@ -871,7 +878,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>travel_rpm_M1</t>
@@ -915,7 +922,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>travel_rpm_M2</t>
@@ -959,7 +966,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>travel_rpm_M3</t>
@@ -1003,7 +1010,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>travel_rpm_M4</t>
@@ -1047,7 +1054,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>torque_travelA</t>
@@ -1091,7 +1098,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>vehicle_speed_encoder</t>
@@ -1135,7 +1142,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>vehicle_speed_gps</t>
@@ -1179,7 +1186,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>position_steerA</t>
@@ -1223,7 +1230,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
+    <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>position_steerB</t>
@@ -1267,7 +1274,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
+    <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>position_steerC</t>
@@ -1311,7 +1318,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>position_steerD</t>
@@ -1355,7 +1362,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1">
+    <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>motor_temp_steerA</t>
@@ -1399,7 +1406,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
+    <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>joystick_cmd_x</t>
@@ -1443,7 +1450,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1">
+    <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>joystick_cmd_y</t>
@@ -1487,7 +1494,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="72" customHeight="1">
+    <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>bms_current</t>
@@ -1531,7 +1538,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1">
+    <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>bms_voltage</t>
@@ -1575,7 +1582,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
+    <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>travel_fault_code_any</t>
@@ -1619,7 +1626,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="48" customHeight="1">
+    <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>operating_mode</t>
@@ -1663,7 +1670,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="36" customHeight="1">
+    <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>distance_m</t>

</xml_diff>